<commit_message>
climate: fix inverted summer label site-wide; correct Memphis and St. Petersburg summer-comfort values
</commit_message>
<xml_diff>
--- a/docs/CityDatabase_Jul_27_v17.xlsx
+++ b/docs/CityDatabase_Jul_27_v17.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="40" windowWidth="15960" windowHeight="18080" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="City Database" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scores by Dimension" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget Tiers" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="New Cities to Add" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parked — Future Build" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="City Database" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Scores by Dimension" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Budget Tiers" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="New Cities to Add" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Parked — Future Build" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -4524,7 +4524,7 @@
         <v>9</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="S30" s="7" t="n">
         <v>8</v>
@@ -9138,7 +9138,7 @@
         <v>5</v>
       </c>
       <c r="R72" s="7" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="S72" s="7" t="n">
         <v>5</v>

</xml_diff>